<commit_message>
Apply QC filtering to COMET NS5A profiles
</commit_message>
<xml_diff>
--- a/Reference_seqs/HCV_Subtype_Ref_vs_Comet_Subtype_Consensus_Aligned_NS5A_NTD.xlsx
+++ b/Reference_seqs/HCV_Subtype_Ref_vs_Comet_Subtype_Consensus_Aligned_NS5A_NTD.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P384"/>
+  <dimension ref="A1:P380"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1305,7 +1305,11 @@
         </is>
       </c>
       <c r="E20" t="inlineStr"/>
-      <c r="F20" t="inlineStr"/>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
       <c r="G20" t="inlineStr"/>
       <c r="H20" t="inlineStr"/>
       <c r="I20" t="inlineStr"/>
@@ -15736,7 +15740,7 @@
       </c>
       <c r="C347" t="inlineStr">
         <is>
-          <t>6u</t>
+          <t>6v</t>
         </is>
       </c>
       <c r="D347" t="inlineStr">
@@ -15746,57 +15750,57 @@
       </c>
       <c r="E347" t="inlineStr">
         <is>
-          <t>K</t>
+          <t>R</t>
         </is>
       </c>
       <c r="F347" t="inlineStr">
         <is>
-          <t>K</t>
+          <t>V</t>
         </is>
       </c>
       <c r="G347" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>S</t>
         </is>
       </c>
       <c r="H347" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>L</t>
         </is>
       </c>
       <c r="I347" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>P</t>
         </is>
       </c>
       <c r="J347" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>G</t>
         </is>
       </c>
       <c r="K347" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>I</t>
         </is>
       </c>
       <c r="L347" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>Q</t>
         </is>
       </c>
       <c r="M347" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>G</t>
         </is>
       </c>
       <c r="N347" t="inlineStr">
         <is>
-          <t>H</t>
+          <t>T</t>
         </is>
       </c>
       <c r="O347" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>T</t>
         </is>
       </c>
       <c r="P347" t="inlineStr">
@@ -15818,7 +15822,7 @@
       </c>
       <c r="C348" t="inlineStr">
         <is>
-          <t>6u</t>
+          <t>6v</t>
         </is>
       </c>
       <c r="D348" t="inlineStr">
@@ -15951,7 +15955,7 @@
       </c>
       <c r="K351" t="inlineStr">
         <is>
-          <t>I</t>
+          <t>V</t>
         </is>
       </c>
       <c r="L351" t="inlineStr">
@@ -16007,7 +16011,11 @@
       <c r="H352" t="inlineStr"/>
       <c r="I352" t="inlineStr"/>
       <c r="J352" t="inlineStr"/>
-      <c r="K352" t="inlineStr"/>
+      <c r="K352" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
       <c r="L352" t="inlineStr"/>
       <c r="M352" t="inlineStr"/>
       <c r="N352" t="inlineStr"/>
@@ -16086,7 +16094,7 @@
       </c>
       <c r="C355" t="inlineStr">
         <is>
-          <t>6v</t>
+          <t>6w</t>
         </is>
       </c>
       <c r="D355" t="inlineStr">
@@ -16096,17 +16104,17 @@
       </c>
       <c r="E355" t="inlineStr">
         <is>
-          <t>R</t>
+          <t>K</t>
         </is>
       </c>
       <c r="F355" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>F</t>
         </is>
       </c>
       <c r="G355" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>A</t>
         </is>
       </c>
       <c r="H355" t="inlineStr">
@@ -16126,7 +16134,7 @@
       </c>
       <c r="K355" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>I</t>
         </is>
       </c>
       <c r="L355" t="inlineStr">
@@ -16141,7 +16149,7 @@
       </c>
       <c r="N355" t="inlineStr">
         <is>
-          <t>T</t>
+          <t>A</t>
         </is>
       </c>
       <c r="O355" t="inlineStr">
@@ -16168,7 +16176,7 @@
       </c>
       <c r="C356" t="inlineStr">
         <is>
-          <t>6v</t>
+          <t>6w</t>
         </is>
       </c>
       <c r="D356" t="inlineStr">
@@ -16177,19 +16185,23 @@
         </is>
       </c>
       <c r="E356" t="inlineStr"/>
-      <c r="F356" t="inlineStr"/>
+      <c r="F356" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
       <c r="G356" t="inlineStr"/>
       <c r="H356" t="inlineStr"/>
       <c r="I356" t="inlineStr"/>
       <c r="J356" t="inlineStr"/>
-      <c r="K356" t="inlineStr">
-        <is>
-          <t>I</t>
-        </is>
-      </c>
+      <c r="K356" t="inlineStr"/>
       <c r="L356" t="inlineStr"/>
       <c r="M356" t="inlineStr"/>
-      <c r="N356" t="inlineStr"/>
+      <c r="N356" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
       <c r="O356" t="inlineStr"/>
       <c r="P356" t="inlineStr"/>
     </row>
@@ -16448,7 +16460,7 @@
       </c>
       <c r="C363" t="inlineStr">
         <is>
-          <t>6w</t>
+          <t>6xa</t>
         </is>
       </c>
       <c r="D363" t="inlineStr">
@@ -16463,12 +16475,12 @@
       </c>
       <c r="F363" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>V</t>
         </is>
       </c>
       <c r="G363" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>S</t>
         </is>
       </c>
       <c r="H363" t="inlineStr">
@@ -16488,7 +16500,7 @@
       </c>
       <c r="K363" t="inlineStr">
         <is>
-          <t>I</t>
+          <t>V</t>
         </is>
       </c>
       <c r="L363" t="inlineStr">
@@ -16503,7 +16515,7 @@
       </c>
       <c r="N363" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>T</t>
         </is>
       </c>
       <c r="O363" t="inlineStr">
@@ -16530,7 +16542,7 @@
       </c>
       <c r="C364" t="inlineStr">
         <is>
-          <t>6w</t>
+          <t>6xa</t>
         </is>
       </c>
       <c r="D364" t="inlineStr">
@@ -16539,11 +16551,7 @@
         </is>
       </c>
       <c r="E364" t="inlineStr"/>
-      <c r="F364" t="inlineStr">
-        <is>
-          <t>V</t>
-        </is>
-      </c>
+      <c r="F364" t="inlineStr"/>
       <c r="G364" t="inlineStr"/>
       <c r="H364" t="inlineStr"/>
       <c r="I364" t="inlineStr"/>
@@ -16551,11 +16559,7 @@
       <c r="K364" t="inlineStr"/>
       <c r="L364" t="inlineStr"/>
       <c r="M364" t="inlineStr"/>
-      <c r="N364" t="inlineStr">
-        <is>
-          <t>T</t>
-        </is>
-      </c>
+      <c r="N364" t="inlineStr"/>
       <c r="O364" t="inlineStr"/>
       <c r="P364" t="inlineStr"/>
     </row>
@@ -16801,12 +16805,12 @@
       </c>
       <c r="B371" t="inlineStr">
         <is>
-          <t>GT6</t>
+          <t>GT7</t>
         </is>
       </c>
       <c r="C371" t="inlineStr">
         <is>
-          <t>6xa</t>
+          <t>7a</t>
         </is>
       </c>
       <c r="D371" t="inlineStr">
@@ -16821,57 +16825,57 @@
       </c>
       <c r="F371" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>K</t>
         </is>
       </c>
       <c r="G371" t="inlineStr">
         <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="H371" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="I371" t="inlineStr">
+        <is>
           <t>S</t>
         </is>
       </c>
-      <c r="H371" t="inlineStr">
+      <c r="J371" t="inlineStr">
         <is>
           <t>L</t>
         </is>
       </c>
-      <c r="I371" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="J371" t="inlineStr">
-        <is>
-          <t>G</t>
-        </is>
-      </c>
       <c r="K371" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>P</t>
         </is>
       </c>
       <c r="L371" t="inlineStr">
         <is>
-          <t>Q</t>
+          <t>S</t>
         </is>
       </c>
       <c r="M371" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>P</t>
         </is>
       </c>
       <c r="N371" t="inlineStr">
         <is>
-          <t>T</t>
+          <t>L</t>
         </is>
       </c>
       <c r="O371" t="inlineStr">
         <is>
-          <t>T</t>
+          <t>S</t>
         </is>
       </c>
       <c r="P371" t="inlineStr">
         <is>
-          <t>T</t>
+          <t>H</t>
         </is>
       </c>
     </row>
@@ -16883,12 +16887,12 @@
       </c>
       <c r="B372" t="inlineStr">
         <is>
-          <t>GT6</t>
+          <t>GT7</t>
         </is>
       </c>
       <c r="C372" t="inlineStr">
         <is>
-          <t>6xa</t>
+          <t>7a</t>
         </is>
       </c>
       <c r="D372" t="inlineStr">
@@ -16981,7 +16985,7 @@
       </c>
       <c r="C375" t="inlineStr">
         <is>
-          <t>7a</t>
+          <t>7b</t>
         </is>
       </c>
       <c r="D375" t="inlineStr">
@@ -17036,12 +17040,12 @@
       </c>
       <c r="N375" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>N</t>
         </is>
       </c>
       <c r="O375" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>A</t>
         </is>
       </c>
       <c r="P375" t="inlineStr">
@@ -17063,7 +17067,7 @@
       </c>
       <c r="C376" t="inlineStr">
         <is>
-          <t>7a</t>
+          <t>7b</t>
         </is>
       </c>
       <c r="D376" t="inlineStr">
@@ -17075,7 +17079,11 @@
       <c r="F376" t="inlineStr"/>
       <c r="G376" t="inlineStr"/>
       <c r="H376" t="inlineStr"/>
-      <c r="I376" t="inlineStr"/>
+      <c r="I376" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
       <c r="J376" t="inlineStr"/>
       <c r="K376" t="inlineStr"/>
       <c r="L376" t="inlineStr"/>
@@ -17151,12 +17159,12 @@
       </c>
       <c r="B379" t="inlineStr">
         <is>
-          <t>GT7</t>
+          <t>GT8</t>
         </is>
       </c>
       <c r="C379" t="inlineStr">
         <is>
-          <t>7b</t>
+          <t>8a</t>
         </is>
       </c>
       <c r="D379" t="inlineStr">
@@ -17171,7 +17179,7 @@
       </c>
       <c r="F379" t="inlineStr">
         <is>
-          <t>K</t>
+          <t>R</t>
         </is>
       </c>
       <c r="G379" t="inlineStr">
@@ -17211,17 +17219,17 @@
       </c>
       <c r="N379" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>V</t>
         </is>
       </c>
       <c r="O379" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>S</t>
         </is>
       </c>
       <c r="P379" t="inlineStr">
         <is>
-          <t>H</t>
+          <t>S</t>
         </is>
       </c>
     </row>
@@ -17233,12 +17241,12 @@
       </c>
       <c r="B380" t="inlineStr">
         <is>
-          <t>GT7</t>
+          <t>GT8</t>
         </is>
       </c>
       <c r="C380" t="inlineStr">
         <is>
-          <t>7b</t>
+          <t>8a</t>
         </is>
       </c>
       <c r="D380" t="inlineStr">
@@ -17247,204 +17255,25 @@
         </is>
       </c>
       <c r="E380" t="inlineStr"/>
-      <c r="F380" t="inlineStr"/>
+      <c r="F380" t="inlineStr">
+        <is>
+          <t>K</t>
+        </is>
+      </c>
       <c r="G380" t="inlineStr"/>
       <c r="H380" t="inlineStr"/>
-      <c r="I380" t="inlineStr">
-        <is>
-          <t>L</t>
-        </is>
-      </c>
+      <c r="I380" t="inlineStr"/>
       <c r="J380" t="inlineStr"/>
       <c r="K380" t="inlineStr"/>
       <c r="L380" t="inlineStr"/>
       <c r="M380" t="inlineStr"/>
-      <c r="N380" t="inlineStr"/>
+      <c r="N380" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
       <c r="O380" t="inlineStr"/>
       <c r="P380" t="inlineStr"/>
-    </row>
-    <row r="381"/>
-    <row r="382">
-      <c r="A382" s="1" t="inlineStr">
-        <is>
-          <t>Gene</t>
-        </is>
-      </c>
-      <c r="B382" s="1" t="inlineStr">
-        <is>
-          <t>Genotype</t>
-        </is>
-      </c>
-      <c r="C382" s="1" t="inlineStr">
-        <is>
-          <t>Subtype</t>
-        </is>
-      </c>
-      <c r="D382" s="1" t="inlineStr">
-        <is>
-          <t>Sequence</t>
-        </is>
-      </c>
-      <c r="E382" s="1" t="n">
-        <v>24</v>
-      </c>
-      <c r="F382" s="1" t="n">
-        <v>26</v>
-      </c>
-      <c r="G382" s="1" t="n">
-        <v>28</v>
-      </c>
-      <c r="H382" s="1" t="n">
-        <v>29</v>
-      </c>
-      <c r="I382" s="1" t="n">
-        <v>30</v>
-      </c>
-      <c r="J382" s="1" t="n">
-        <v>31</v>
-      </c>
-      <c r="K382" s="1" t="n">
-        <v>32</v>
-      </c>
-      <c r="L382" s="1" t="n">
-        <v>38</v>
-      </c>
-      <c r="M382" s="1" t="n">
-        <v>58</v>
-      </c>
-      <c r="N382" s="1" t="n">
-        <v>62</v>
-      </c>
-      <c r="O382" s="1" t="n">
-        <v>92</v>
-      </c>
-      <c r="P382" s="1" t="n">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="383">
-      <c r="A383" t="inlineStr">
-        <is>
-          <t>NS5A_NTD</t>
-        </is>
-      </c>
-      <c r="B383" t="inlineStr">
-        <is>
-          <t>GT8</t>
-        </is>
-      </c>
-      <c r="C383" t="inlineStr">
-        <is>
-          <t>8a</t>
-        </is>
-      </c>
-      <c r="D383" t="inlineStr">
-        <is>
-          <t>Reference</t>
-        </is>
-      </c>
-      <c r="E383" t="inlineStr">
-        <is>
-          <t>K</t>
-        </is>
-      </c>
-      <c r="F383" t="inlineStr">
-        <is>
-          <t>R</t>
-        </is>
-      </c>
-      <c r="G383" t="inlineStr">
-        <is>
-          <t>L</t>
-        </is>
-      </c>
-      <c r="H383" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="I383" t="inlineStr">
-        <is>
-          <t>S</t>
-        </is>
-      </c>
-      <c r="J383" t="inlineStr">
-        <is>
-          <t>L</t>
-        </is>
-      </c>
-      <c r="K383" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="L383" t="inlineStr">
-        <is>
-          <t>S</t>
-        </is>
-      </c>
-      <c r="M383" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="N383" t="inlineStr">
-        <is>
-          <t>V</t>
-        </is>
-      </c>
-      <c r="O383" t="inlineStr">
-        <is>
-          <t>S</t>
-        </is>
-      </c>
-      <c r="P383" t="inlineStr">
-        <is>
-          <t>S</t>
-        </is>
-      </c>
-    </row>
-    <row r="384">
-      <c r="A384" t="inlineStr">
-        <is>
-          <t>NS5A_NTD</t>
-        </is>
-      </c>
-      <c r="B384" t="inlineStr">
-        <is>
-          <t>GT8</t>
-        </is>
-      </c>
-      <c r="C384" t="inlineStr">
-        <is>
-          <t>8a</t>
-        </is>
-      </c>
-      <c r="D384" t="inlineStr">
-        <is>
-          <t>Consensus</t>
-        </is>
-      </c>
-      <c r="E384" t="inlineStr"/>
-      <c r="F384" t="inlineStr">
-        <is>
-          <t>K</t>
-        </is>
-      </c>
-      <c r="G384" t="inlineStr"/>
-      <c r="H384" t="inlineStr"/>
-      <c r="I384" t="inlineStr"/>
-      <c r="J384" t="inlineStr"/>
-      <c r="K384" t="inlineStr"/>
-      <c r="L384" t="inlineStr"/>
-      <c r="M384" t="inlineStr"/>
-      <c r="N384" t="inlineStr">
-        <is>
-          <t>I</t>
-        </is>
-      </c>
-      <c r="O384" t="inlineStr"/>
-      <c r="P384" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>